<commit_message>
Add uploaded OCHA figures (Excel) for South_Sudan___SSD
</commit_message>
<xml_diff>
--- a/platform_PiN_output/South_Sudan___SSD/ocha_figures_South_Sudan___SSD_1028_03PM.xlsx
+++ b/platform_PiN_output/South_Sudan___SSD/ocha_figures_South_Sudan___SSD_1028_03PM.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ocha_data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="mismatch_ocha_data" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3254,786 +3253,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C80"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">List of admin-pcode where MSNA data is representative at the unit of analysis of the HNO (e.g. if your analysis is conducted at admin 3, include the list of admin/pcode where the data is representative at admin 3) ----  Liste des codes admin où les données MSNA sont représentatives à l'unité d'analyse de l'HNO (par exemple, si votre analyse est effectuée à l'admin 3, incluez la liste des codes admin où les données sont représentatives à l'admin 3) </t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>List of admin-pcode where MSNA data is not representative at the unit of analysis of the HNO (e.g., if your analysis is conducted at admin 3, but in some admin 3 units the data is only representative at admin 2 -&gt; include these admin 3 units) ---- Liste des codes admin où les données MSNA ne sont pas représentatives à l'unité d'analyse de la HNO (par exemple, si votre analyse est effectuée à l'admin 3, mais que dans certaines unités de l'admin 3 les données ne sont représentatives qu'à l'admin 2 -&gt; inclure ces unités de l'admin 3).</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Unique list of admin codes at one or more levels above OCHA's unit of analysis that are representative in the MSNA and present in the MSNA data. ---- Liste unique de codes administratifs à un ou plusieurs niveaux au-dessus de l'unité d'analyse d'OCHA qui sont représentatifs dans le MSNA et présents dans les données du MSNA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SS0001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>SS01</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SS0101</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>SS02</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>SS0102</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>SS03</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SS0103</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SS04</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>SS0104</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SS05</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>SS0105</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SS06</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>SS0106</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>SS07</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>SS0201</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>SS08</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr"/>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>SS0202</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>SS09</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>SS0203</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>SS10</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>SS0204</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>SS0205</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>SS0206</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>SS0207</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>SS0208</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>SS0301</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr"/>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SS0302</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>SS0303</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>SS0304</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>SS0305</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>SS0306</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>SS0307</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>SS0308</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>SS0309</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr"/>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>SS0310</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>SS0311</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>SS0401</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>SS0402</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr"/>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>SS0403</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr"/>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>SS0404</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr"/>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>SS0405</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr"/>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>SS0406</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>SS0407</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>SS0408</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr"/>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>SS0501</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>SS0502</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr"/>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>SS0503</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>SS0504</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SS0505</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr"/>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>SS0601</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr"/>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>SS0602</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr"/>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>SS0603</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr"/>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>SS0604</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr"/>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>SS0605</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr"/>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>SS0606</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>SS0607</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>SS0608</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr"/>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>SS0609</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>SS0701</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>SS0702</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr"/>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>SS0703</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr"/>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>SS0704</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr"/>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>SS0705</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>SS0706</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr"/>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>SS0707</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr"/>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>SS0708</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr"/>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>SS0709</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr"/>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>SS0710</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr"/>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>SS0711</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr"/>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>SS0712</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr"/>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>SS0801</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr"/>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>SS0802</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr"/>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>SS0803</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr"/>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>SS0804</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr"/>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>SS0805</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr"/>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>SS0806</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr"/>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>SS0901</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr"/>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>SS0902</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr"/>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>SS0903</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr"/>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>SS1001</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr"/>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>SS1002</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr"/>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>SS1003</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr"/>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>SS1004</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr"/>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>SS1005</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr"/>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>SS1006</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr"/>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>SS1007</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr"/>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>SS1008</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr"/>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>SS1009</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr"/>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>SS1010</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>